<commit_message>
Realistic statuses, on-time by analyst and team, SQL Server, run_all
</commit_message>
<xml_diff>
--- a/output/request_summary.xlsx
+++ b/output/request_summary.xlsx
@@ -10,13 +10,15 @@
     <sheet name="KPIs" sheetId="1" r:id="rId1"/>
     <sheet name="By team" sheetId="2" r:id="rId2"/>
     <sheet name="Monthly volume" sheetId="3" r:id="rId3"/>
+    <sheet name="On time by analyst" sheetId="4" r:id="rId4"/>
+    <sheet name="On time by team" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="26">
   <si>
     <t>Metric</t>
   </si>
@@ -48,12 +50,12 @@
     <t>team</t>
   </si>
   <si>
+    <t>Operations</t>
+  </si>
+  <si>
     <t>Finance</t>
   </si>
   <si>
-    <t>Operations</t>
-  </si>
-  <si>
     <t>Sales</t>
   </si>
   <si>
@@ -76,6 +78,24 @@
   </si>
   <si>
     <t>2026-09</t>
+  </si>
+  <si>
+    <t>completed</t>
+  </si>
+  <si>
+    <t>on_time_pct</t>
+  </si>
+  <si>
+    <t>assigned_to</t>
+  </si>
+  <si>
+    <t>Analyst B</t>
+  </si>
+  <si>
+    <t>Analyst A</t>
+  </si>
+  <si>
+    <t>Analyst C</t>
   </si>
 </sst>
 </file>
@@ -431,7 +451,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>228</v>
+        <v>279</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -439,7 +459,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>72</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -455,7 +475,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>2.1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -484,7 +504,7 @@
         <v>10</v>
       </c>
       <c r="B2">
-        <v>64</v>
+        <v>81</v>
       </c>
       <c r="C2">
         <v>2.3</v>
@@ -495,10 +515,10 @@
         <v>11</v>
       </c>
       <c r="B3">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="C3">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -506,10 +526,10 @@
         <v>12</v>
       </c>
       <c r="B4">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="C4">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -517,10 +537,10 @@
         <v>13</v>
       </c>
       <c r="B5">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C5">
-        <v>2.8</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -528,10 +548,10 @@
         <v>14</v>
       </c>
       <c r="B6">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="C6">
-        <v>2.6</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -555,10 +575,10 @@
         <v>13</v>
       </c>
       <c r="D1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" t="s">
         <v>10</v>
-      </c>
-      <c r="E1" t="s">
-        <v>11</v>
       </c>
       <c r="F1" t="s">
         <v>12</v>
@@ -569,19 +589,19 @@
         <v>16</v>
       </c>
       <c r="B2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2">
         <v>7</v>
       </c>
       <c r="D2">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E2">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F2">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -589,7 +609,7 @@
         <v>17</v>
       </c>
       <c r="B3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C3">
         <v>6</v>
@@ -598,7 +618,7 @@
         <v>25</v>
       </c>
       <c r="E3">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F3">
         <v>13</v>
@@ -612,16 +632,16 @@
         <v>8</v>
       </c>
       <c r="C4">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D4">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E4">
         <v>16</v>
       </c>
       <c r="F4">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -629,19 +649,149 @@
         <v>19</v>
       </c>
       <c r="B5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C5">
+        <v>13</v>
+      </c>
+      <c r="D5">
+        <v>20</v>
+      </c>
+      <c r="E5">
+        <v>27</v>
+      </c>
+      <c r="F5">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2">
+        <v>77</v>
+      </c>
+      <c r="C2">
+        <v>46.8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3">
+        <v>94</v>
+      </c>
+      <c r="C3">
+        <v>78.7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4">
+        <v>108</v>
+      </c>
+      <c r="C4">
+        <v>81.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
         <v>14</v>
       </c>
-      <c r="D5">
-        <v>18</v>
-      </c>
-      <c r="E5">
+      <c r="B2">
+        <v>26</v>
+      </c>
+      <c r="C2">
+        <v>57.7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3">
+        <v>77</v>
+      </c>
+      <c r="C3">
+        <v>66.2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>81</v>
+      </c>
+      <c r="C4">
+        <v>67.90000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5">
         <v>29</v>
       </c>
-      <c r="F5">
-        <v>23</v>
+      <c r="C5">
+        <v>72.40000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6">
+        <v>66</v>
+      </c>
+      <c r="C6">
+        <v>84.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>